<commit_message>
Refactor algorithm and exporter; add tests and update input data
- algorithm.py: rewrite distribution logic with priority phases and zero-residue guarantee
- exporter.py: expand Excel output to 3 sheets with full formatting
- tests: add test_algorithm.py coverage and new test_exporter.py
- app.py / run.py: minor fixes
- Input/: update source Excel files to latest data
- CLAUDE.md: document implementation details and known doc contradiction

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Input/Tiendas_No generar pedido.xlsx
+++ b/Input/Tiendas_No generar pedido.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prestamo\Documents\Isimo\Proyectos\Distribucion de Fruver\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9B80EF1-9E5E-4D90-9BE5-09B6A6EC3890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7825B37-4420-44FA-8336-EF6A1F436F31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="15375" windowHeight="7875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Update Input data files
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Input/Tiendas_No generar pedido.xlsx
+++ b/Input/Tiendas_No generar pedido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prestamo\Documents\Isimo\Proyectos\Distribucion de Fruver\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7825B37-4420-44FA-8336-EF6A1F436F31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44035C6E-9F9E-4C52-93AC-EB439C937C94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Centro Operacional de la Bodega</t>
   </si>
@@ -45,6 +45,33 @@
   </si>
   <si>
     <t>ISIMO TO GO</t>
+  </si>
+  <si>
+    <t>S17</t>
+  </si>
+  <si>
+    <t>S18</t>
+  </si>
+  <si>
+    <t>S34</t>
+  </si>
+  <si>
+    <t>S70</t>
+  </si>
+  <si>
+    <t>S83</t>
+  </si>
+  <si>
+    <t>SA5</t>
+  </si>
+  <si>
+    <t>SE8</t>
+  </si>
+  <si>
+    <t>S31</t>
+  </si>
+  <si>
+    <t>SA6</t>
   </si>
 </sst>
 </file>
@@ -413,7 +440,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="13.5703125" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="28.5703125" bestFit="1" customWidth="1"/>
@@ -433,17 +460,50 @@
       </c>
     </row>
     <row r="3" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="1"/>
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
       <c r="B3" s="2"/>
     </row>
+    <row r="4" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+    </row>
     <row r="5" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="1"/>
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="6" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="1"/>
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="7" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="1"/>
+      <c r="A7" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>